<commit_message>
Made Fetch 1 Stage
</commit_message>
<xml_diff>
--- a/proj1/microcode.xlsx
+++ b/proj1/microcode.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="111">
   <si>
     <t xml:space="preserve">Index</t>
   </si>
@@ -106,16 +106,10 @@
     <t xml:space="preserve">Comment</t>
   </si>
   <si>
-    <t xml:space="preserve">Fetch0</t>
+    <t xml:space="preserve">FETCH</t>
   </si>
   <si>
     <t xml:space="preserve">NULL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fetch1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fetch2</t>
   </si>
   <si>
     <t xml:space="preserve">Halt</t>
@@ -830,37 +824,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Sheets">
@@ -1006,7 +1000,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="3" style="1" width="2.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="2.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="9.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="13" style="1" width="9.5"/>
@@ -1149,14 +1143,14 @@
         <v>0</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="8" t="n">
         <f aca="false">BIN2DEC(_xlfn.CONCAT(C2:H2))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -1183,22 +1177,22 @@
         <v>0</v>
       </c>
       <c r="R2" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T2" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="W2" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X2" s="5" t="n">
         <v>0</v>
@@ -1222,12 +1216,12 @@
         <v>0</v>
       </c>
       <c r="AE2" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF2" s="7"/>
       <c r="AG2" s="9" t="str">
         <f aca="false">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(J2, K2, L2, M2),1),     BIN2HEX(_xlfn.CONCAT(N2,O2,P2,Q2),1),     BIN2HEX(_xlfn.CONCAT(R2,S2,T2,U2),1),     BIN2HEX(_xlfn.CONCAT(V2,W2,X2,Y2),1),     BIN2HEX(_xlfn.CONCAT(Z2,AA2,AB2,AC2),1),     BIN2HEX(_xlfn.CONCAT(AD2,AE2,C2,D2),1),     BIN2HEX(_xlfn.CONCAT(E2,F2,G2,H2),1) )</f>
-        <v>00C4002</v>
+        <v>0030040</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1250,14 +1244,14 @@
         <v>0</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="8" t="n">
         <f aca="false">BIN2DEC(_xlfn.CONCAT(C3:H3))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>0</v>
@@ -1284,10 +1278,10 @@
         <v>0</v>
       </c>
       <c r="R3" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T3" s="5" t="n">
         <v>0</v>
@@ -1299,7 +1293,7 @@
         <v>0</v>
       </c>
       <c r="W3" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X3" s="5" t="n">
         <v>0</v>
@@ -1328,7 +1322,7 @@
       <c r="AF3" s="7"/>
       <c r="AG3" s="9" t="str">
         <f aca="false">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(J3, K3, L3, M3),1),     BIN2HEX(_xlfn.CONCAT(N3,O3,P3,Q3),1),     BIN2HEX(_xlfn.CONCAT(R3,S3,T3,U3),1),     BIN2HEX(_xlfn.CONCAT(V3,W3,X3,Y3),1),     BIN2HEX(_xlfn.CONCAT(Z3,AA3,AB3,AC3),1),     BIN2HEX(_xlfn.CONCAT(AD3,AE3,C3,D3),1),     BIN2HEX(_xlfn.CONCAT(E3,F3,G3,H3),1) )</f>
-        <v>00C4002</v>
+        <v>0000000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1336,7 +1330,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>0</v>
@@ -1351,14 +1345,14 @@
         <v>0</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="8" t="n">
         <f aca="false">BIN2DEC(_xlfn.CONCAT(C4:H4))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -1391,7 +1385,7 @@
         <v>0</v>
       </c>
       <c r="T4" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U4" s="5" t="n">
         <v>0</v>
@@ -1406,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="5" t="n">
         <v>0</v>
@@ -1429,7 +1423,7 @@
       <c r="AF4" s="7"/>
       <c r="AG4" s="9" t="str">
         <f aca="false">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(J4, K4, L4, M4),1),     BIN2HEX(_xlfn.CONCAT(N4,O4,P4,Q4),1),     BIN2HEX(_xlfn.CONCAT(R4,S4,T4,U4),1),     BIN2HEX(_xlfn.CONCAT(V4,W4,X4,Y4),1),     BIN2HEX(_xlfn.CONCAT(Z4,AA4,AB4,AC4),1),     BIN2HEX(_xlfn.CONCAT(AD4,AE4,C4,D4),1),     BIN2HEX(_xlfn.CONCAT(E4,F4,G4,H4),1) )</f>
-        <v>0021003</v>
+        <v>0000000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1438,7 +1432,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>0</v>
@@ -1472,10 +1466,10 @@
         <v>0</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" s="5" t="n">
         <v>0</v>
@@ -1496,7 +1490,7 @@
         <v>0</v>
       </c>
       <c r="U5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V5" s="5" t="n">
         <v>0</v>
@@ -1505,7 +1499,7 @@
         <v>0</v>
       </c>
       <c r="X5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="5" t="n">
         <v>0</v>
@@ -1526,12 +1520,12 @@
         <v>0</v>
       </c>
       <c r="AE5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF5" s="7"/>
       <c r="AG5" s="9" t="str">
         <f aca="false">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(J5, K5, L5, M5),1),     BIN2HEX(_xlfn.CONCAT(N5,O5,P5,Q5),1),     BIN2HEX(_xlfn.CONCAT(R5,S5,T5,U5),1),     BIN2HEX(_xlfn.CONCAT(V5,W5,X5,Y5),1),     BIN2HEX(_xlfn.CONCAT(Z5,AA5,AB5,AC5),1),     BIN2HEX(_xlfn.CONCAT(AD5,AE5,C5,D5),1),     BIN2HEX(_xlfn.CONCAT(E5,F5,G5,H5),1) )</f>
-        <v>1812040</v>
+        <v>0000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1540,7 +1534,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>0</v>
@@ -1613,7 +1607,7 @@
         <v>0</v>
       </c>
       <c r="Z6" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="5" t="n">
         <v>0</v>
@@ -1633,7 +1627,7 @@
       <c r="AF6" s="7"/>
       <c r="AG6" s="9" t="str">
         <f aca="false">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(J6, K6, L6, M6),1),     BIN2HEX(_xlfn.CONCAT(N6,O6,P6,Q6),1),     BIN2HEX(_xlfn.CONCAT(R6,S6,T6,U6),1),     BIN2HEX(_xlfn.CONCAT(V6,W6,X6,Y6),1),     BIN2HEX(_xlfn.CONCAT(Z6,AA6,AB6,AC6),1),     BIN2HEX(_xlfn.CONCAT(AD6,AE6,C6,D6),1),     BIN2HEX(_xlfn.CONCAT(E6,F6,G6,H6),1) )</f>
-        <v>0000804</v>
+        <v>0000004</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1642,7 +1636,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>0</v>
@@ -1744,7 +1738,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>0</v>
@@ -1846,7 +1840,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>0</v>
@@ -1948,7 +1942,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>0</v>
@@ -2021,7 +2015,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA10" s="5" t="n">
         <v>0</v>
@@ -2041,7 +2035,7 @@
       <c r="AF10" s="7"/>
       <c r="AG10" s="9" t="str">
         <f aca="false">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(J10, K10, L10, M10),1),     BIN2HEX(_xlfn.CONCAT(N10,O10,P10,Q10),1),     BIN2HEX(_xlfn.CONCAT(R10,S10,T10,U10),1),     BIN2HEX(_xlfn.CONCAT(V10,W10,X10,Y10),1),     BIN2HEX(_xlfn.CONCAT(Z10,AA10,AB10,AC10),1),     BIN2HEX(_xlfn.CONCAT(AD10,AE10,C10,D10),1),     BIN2HEX(_xlfn.CONCAT(E10,F10,G10,H10),1) )</f>
-        <v>4080009</v>
+        <v>4080809</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2050,7 +2044,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>0</v>
@@ -2152,7 +2146,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>0</v>
@@ -2254,7 +2248,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>0</v>
@@ -2350,13 +2344,13 @@
         <v>408080C</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="n">
         <f aca="false">A13+1</f>
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>0</v>
@@ -2458,7 +2452,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
@@ -2560,7 +2554,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C16" s="5" t="n">
         <v>0</v>
@@ -2662,7 +2656,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
@@ -2764,7 +2758,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>0</v>
@@ -2866,7 +2860,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
@@ -2968,7 +2962,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C20" s="5" t="n">
         <v>0</v>
@@ -3070,7 +3064,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>0</v>
@@ -3172,7 +3166,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
@@ -3274,7 +3268,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>0</v>
@@ -3376,7 +3370,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
@@ -3478,7 +3472,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C25" s="5" t="n">
         <v>0</v>
@@ -3580,7 +3574,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>0</v>
@@ -3682,7 +3676,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>0</v>
@@ -3784,7 +3778,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>0</v>
@@ -3886,7 +3880,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>0</v>
@@ -3988,7 +3982,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>0</v>
@@ -4090,7 +4084,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>0</v>
@@ -4192,7 +4186,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>0</v>
@@ -4294,7 +4288,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>1</v>
@@ -4396,7 +4390,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
@@ -4498,7 +4492,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C35" s="5" t="n">
         <v>1</v>
@@ -4600,7 +4594,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>1</v>
@@ -4702,7 +4696,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>0</v>
@@ -4804,7 +4798,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C38" s="5" t="n">
         <v>1</v>
@@ -4906,7 +4900,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C39" s="5" t="n">
         <v>1</v>
@@ -5002,7 +4996,7 @@
         <v>8100826</v>
       </c>
       <c r="AH39" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5011,7 +5005,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C40" s="5" t="n">
         <v>1</v>
@@ -5113,7 +5107,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C41" s="5" t="n">
         <v>0</v>
@@ -5215,7 +5209,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C42" s="5" t="n">
         <v>0</v>
@@ -5317,7 +5311,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C43" s="5" t="n">
         <v>1</v>
@@ -5419,7 +5413,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C44" s="5" t="n">
         <v>1</v>
@@ -5521,7 +5515,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C45" s="5" t="n">
         <v>1</v>
@@ -7624,7 +7618,7 @@
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
@@ -7635,13 +7629,13 @@
       <c r="I68" s="10"/>
       <c r="J68" s="10"/>
       <c r="L68" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M68" s="10"/>
       <c r="N68" s="10"/>
       <c r="O68" s="10"/>
       <c r="Q68" s="11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="R68" s="11"/>
       <c r="S68" s="11"/>
@@ -7650,10 +7644,10 @@
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="13"/>
@@ -7664,19 +7658,19 @@
         <v>27</v>
       </c>
       <c r="J69" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="L69" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="M69" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="L69" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="M69" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="N69" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="O69" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="Q69" s="11"/>
       <c r="R69" s="11"/>
@@ -7686,10 +7680,10 @@
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C70" s="16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D70" s="16"/>
       <c r="E70" s="16"/>
@@ -7697,17 +7691,17 @@
       <c r="G70" s="16"/>
       <c r="H70" s="16"/>
       <c r="I70" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J70" s="17" t="str">
         <f aca="false">DEC2HEX(C70)</f>
         <v>19</v>
       </c>
       <c r="L70" s="18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="M70" s="19" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N70" s="7" t="n">
         <v>5</v>
@@ -7724,10 +7718,10 @@
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C71" s="16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D71" s="16"/>
       <c r="E71" s="16"/>
@@ -7735,17 +7729,17 @@
       <c r="G71" s="16"/>
       <c r="H71" s="16"/>
       <c r="I71" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J71" s="17" t="str">
         <f aca="false">DEC2HEX(C71)</f>
         <v>27</v>
       </c>
       <c r="L71" s="18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="M71" s="19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="N71" s="7" t="n">
         <v>8</v>
@@ -7774,10 +7768,10 @@
         <v>0</v>
       </c>
       <c r="L72" s="18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="M72" s="19" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="N72" s="7" t="n">
         <v>11</v>
@@ -7806,10 +7800,10 @@
         <v>0</v>
       </c>
       <c r="L73" s="18" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M73" s="19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="N73" s="7" t="n">
         <v>14</v>
@@ -7833,10 +7827,10 @@
       <c r="H74" s="19"/>
       <c r="I74" s="5"/>
       <c r="L74" s="18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="M74" s="19" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="N74" s="7" t="n">
         <v>18</v>
@@ -7848,10 +7842,10 @@
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L75" s="18" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M75" s="19" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="N75" s="7" t="n">
         <v>22</v>
@@ -7861,7 +7855,7 @@
         <v>16</v>
       </c>
       <c r="Q75" s="24" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="R75" s="24"/>
       <c r="S75" s="24"/>
@@ -7870,10 +7864,10 @@
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L76" s="18" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M76" s="19" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="N76" s="7" t="n">
         <v>28</v>
@@ -7890,10 +7884,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L77" s="18" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="M77" s="19" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="N77" s="7" t="n">
         <v>4</v>
@@ -7910,10 +7904,10 @@
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L78" s="18" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="M78" s="19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N78" s="7" t="n">
         <v>30</v>
@@ -7930,10 +7924,10 @@
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L79" s="18" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="M79" s="19" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N79" s="7" t="n">
         <v>33</v>
@@ -7950,10 +7944,10 @@
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L80" s="18" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M80" s="19" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N80" s="7" t="n">
         <v>36</v>
@@ -7970,10 +7964,10 @@
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L81" s="18" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="M81" s="19" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="N81" s="7" t="n">
         <v>41</v>
@@ -8023,7 +8017,7 @@
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="L87" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="M87" s="26"/>
       <c r="N87" s="26"/>
@@ -8994,7 +8988,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:H19">
+  <conditionalFormatting sqref="C3:H19 C3:H19 C3:H19 C3:H19">
     <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>1</formula>
     </cfRule>
@@ -9003,94 +8997,62 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:H19">
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:H19">
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:H19">
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>LEN(TRIM(C3))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:H19">
-    <cfRule type="cellIs" priority="14" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+  <conditionalFormatting sqref="C4:H18">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4:H18">
-    <cfRule type="cellIs" priority="16" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="17" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:H2">
-    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:H2">
-    <cfRule type="cellIs" priority="19" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="20" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="cellIs" priority="14" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:H18 C3:H18">
+    <cfRule type="cellIs" priority="15" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="16" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:H18">
-    <cfRule type="cellIs" priority="21" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="22" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:H18">
-    <cfRule type="cellIs" priority="23" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="24" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:H18">
-    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>LEN(TRIM(C3))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:H18">
-    <cfRule type="cellIs" priority="26" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+    <cfRule type="cellIs" priority="18" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="27" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="cellIs" priority="19" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L25">
-    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>LEN(TRIM(L26))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L25">
-    <cfRule type="cellIs" priority="29" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="21" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="30" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="cellIs" priority="22" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>